<commit_message>
Revert "Merge branch 'main' of https://github.com/Thelia-Lzr/BoomJam26"
This reverts commit 668b70d4e9857a9d06a461c24e85fbb999735ee2, reversing
changes made to 415c924a97db83ccd30ff74cdb0e31e3f1880c06.
</commit_message>
<xml_diff>
--- a/Assets/Resource/Q/QDialogue.xlsx
+++ b/Assets/Resource/Q/QDialogue.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="30">
   <si>
     <t>segmentId</t>
   </si>
@@ -119,18 +119,6 @@
   </si>
   <si>
     <t>加油。</t>
-  </si>
-  <si>
-    <t>哦对了。</t>
-  </si>
-  <si>
-    <t>你可以通过“W”“A”“S”“D”控制视野。</t>
-  </si>
-  <si>
-    <t>另外还可以把已部署的框拖拽到屏幕最下边来删除这个框。</t>
-  </si>
-  <si>
-    <t>祝你好运！</t>
   </si>
 </sst>
 </file>
@@ -1064,7 +1052,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="4" max="4" width="37.6666666666667" customWidth="1"/>
@@ -1355,75 +1343,7 @@
       <c r="D17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="1">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="1">
-        <v>5</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="1">
-        <v>6</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D20" t="s">
-        <v>32</v>
-      </c>
-      <c r="E20" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B21" s="1">
-        <v>7</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="E17" s="1" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reapply "Merge branch 'main' of https://github.com/Thelia-Lzr/BoomJam26"
This reverts commit de2eac6695c5391715102c373ca81722f8e20987.
</commit_message>
<xml_diff>
--- a/Assets/Resource/Q/QDialogue.xlsx
+++ b/Assets/Resource/Q/QDialogue.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="34">
   <si>
     <t>segmentId</t>
   </si>
@@ -119,6 +119,18 @@
   </si>
   <si>
     <t>加油。</t>
+  </si>
+  <si>
+    <t>哦对了。</t>
+  </si>
+  <si>
+    <t>你可以通过“W”“A”“S”“D”控制视野。</t>
+  </si>
+  <si>
+    <t>另外还可以把已部署的框拖拽到屏幕最下边来删除这个框。</t>
+  </si>
+  <si>
+    <t>祝你好运！</t>
   </si>
 </sst>
 </file>
@@ -1052,7 +1064,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="4" max="4" width="37.6666666666667" customWidth="1"/>
@@ -1343,7 +1355,75 @@
       <c r="D17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="1">
+        <v>4</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="1">
+        <v>5</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="1">
+        <v>6</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="1">
+        <v>7</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>